<commit_message>
add manual map and code to process kmz files
</commit_message>
<xml_diff>
--- a/List_villages.xlsx
+++ b/List_villages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/859d9643ad450da0/Recherche/Projet émergent/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\solar-data-china\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{738D009E-1742-4692-9867-79C853F44E2A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B69048-D6B0-4976-ACB7-B9ACF5DB1CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="6563" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="494">
   <si>
     <t>Province</t>
   </si>
@@ -1496,13 +1496,22 @@
   </si>
   <si>
     <t>张家口市</t>
+  </si>
+  <si>
+    <t>https://www.google.fr/maps/d/u/0/edit?mid=18TO9l56bvv5GElt6nxTtLuWsAZPKIDY&amp;usp=sharing</t>
+  </si>
+  <si>
+    <t>https://www.google.fr/maps/d/u/0/edit?mid=1wB8JRtKsavhiC53-NBhw93nwuybg1ss&amp;usp=sharing</t>
+  </si>
+  <si>
+    <t>https://www.google.fr/maps/d/u/0/edit?mid=13pRx0pCU6D9YJSQszlKe2FWlEIxfusI&amp;usp=sharing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1514,6 +1523,15 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1524,7 +1542,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1547,11 +1565,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1572,8 +1600,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1874,25 +1909,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M112"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:N112"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.06640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1328125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.265625" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.73046875" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.19921875" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.1328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.9296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.9296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.19921875" style="7" customWidth="1"/>
-    <col min="11" max="11" width="20.19921875" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.21875" style="7" customWidth="1"/>
+    <col min="11" max="11" width="20.21875" style="7" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19" style="7" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="29.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="74.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1933,7 +1969,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>207</v>
       </c>
@@ -1973,8 +2009,11 @@
       <c r="M2" s="6" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N2" s="8" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>207</v>
       </c>
@@ -2014,8 +2053,9 @@
       <c r="M3" s="6" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N3" s="9"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>207</v>
       </c>
@@ -2055,8 +2095,9 @@
       <c r="M4" s="6" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N4" s="9"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>207</v>
       </c>
@@ -2096,8 +2137,9 @@
       <c r="M5" s="6" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N5" s="9"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>207</v>
       </c>
@@ -2137,8 +2179,9 @@
       <c r="M6" s="6" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>207</v>
       </c>
@@ -2178,8 +2221,9 @@
       <c r="M7" s="6" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N7" s="9"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>207</v>
       </c>
@@ -2219,8 +2263,9 @@
       <c r="M8" s="6" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N8" s="9"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>207</v>
       </c>
@@ -2260,8 +2305,9 @@
       <c r="M9" s="6" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N9" s="9"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>207</v>
       </c>
@@ -2301,8 +2347,9 @@
       <c r="M10" s="6" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N10" s="9"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>207</v>
       </c>
@@ -2342,8 +2389,9 @@
       <c r="M11" s="6" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N11" s="9"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>207</v>
       </c>
@@ -2383,8 +2431,11 @@
       <c r="M12" s="6" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N12" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>207</v>
       </c>
@@ -2424,8 +2475,9 @@
       <c r="M13" s="6" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N13" s="9"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>207</v>
       </c>
@@ -2465,8 +2517,9 @@
       <c r="M14" s="6" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N14" s="9"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>207</v>
       </c>
@@ -2506,8 +2559,9 @@
       <c r="M15" s="6" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N15" s="9"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>207</v>
       </c>
@@ -2547,8 +2601,9 @@
       <c r="M16" s="6" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N16" s="9"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>207</v>
       </c>
@@ -2588,8 +2643,9 @@
       <c r="M17" s="6" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N17" s="9"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>207</v>
       </c>
@@ -2629,8 +2685,9 @@
       <c r="M18" s="6" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N18" s="9"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>207</v>
       </c>
@@ -2670,8 +2727,9 @@
       <c r="M19" s="6" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N19" s="9"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>207</v>
       </c>
@@ -2711,8 +2769,9 @@
       <c r="M20" s="6" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N20" s="9"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>115</v>
       </c>
@@ -2752,8 +2811,9 @@
       <c r="M21" s="6" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N21" s="9"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>115</v>
       </c>
@@ -2793,8 +2853,9 @@
       <c r="M22" s="6" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N22" s="9"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>115</v>
       </c>
@@ -2834,8 +2895,9 @@
       <c r="M23" s="6" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N23" s="9"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>115</v>
       </c>
@@ -2875,8 +2937,9 @@
       <c r="M24" s="6" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N24" s="9"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>115</v>
       </c>
@@ -2916,8 +2979,9 @@
       <c r="M25" s="6" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N25" s="9"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>115</v>
       </c>
@@ -2957,8 +3021,11 @@
       <c r="M26" s="6" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N26" s="8" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>115</v>
       </c>
@@ -2998,8 +3065,9 @@
       <c r="M27" s="6" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N27" s="9"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>115</v>
       </c>
@@ -3039,8 +3107,9 @@
       <c r="M28" s="6" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N28" s="9"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>115</v>
       </c>
@@ -3080,8 +3149,9 @@
       <c r="M29" s="6" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N29" s="9"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>115</v>
       </c>
@@ -3121,8 +3191,9 @@
       <c r="M30" s="6" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N30" s="9"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>115</v>
       </c>
@@ -3162,8 +3233,9 @@
       <c r="M31" s="6" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N31" s="9"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>115</v>
       </c>
@@ -3203,8 +3275,9 @@
       <c r="M32" s="6" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N32" s="9"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>115</v>
       </c>
@@ -3244,8 +3317,9 @@
       <c r="M33" s="6" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N33" s="9"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>115</v>
       </c>
@@ -3285,8 +3359,9 @@
       <c r="M34" s="6" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N34" s="9"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>115</v>
       </c>
@@ -3326,8 +3401,9 @@
       <c r="M35" s="6" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N35" s="9"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>115</v>
       </c>
@@ -3367,8 +3443,9 @@
       <c r="M36" s="6" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N36" s="9"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>115</v>
       </c>
@@ -3408,8 +3485,9 @@
       <c r="M37" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N37" s="9"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>115</v>
       </c>
@@ -3449,8 +3527,9 @@
       <c r="M38" s="6" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N38" s="9"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>115</v>
       </c>
@@ -3490,8 +3569,9 @@
       <c r="M39" s="6" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N39" s="9"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>115</v>
       </c>
@@ -3532,7 +3612,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>115</v>
       </c>
@@ -3573,7 +3653,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>115</v>
       </c>
@@ -3614,7 +3694,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>115</v>
       </c>
@@ -3655,7 +3735,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>115</v>
       </c>
@@ -3696,7 +3776,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>115</v>
       </c>
@@ -3737,7 +3817,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>115</v>
       </c>
@@ -3778,7 +3858,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>281</v>
       </c>
@@ -3819,7 +3899,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>281</v>
       </c>
@@ -3860,7 +3940,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>281</v>
       </c>
@@ -3901,7 +3981,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>281</v>
       </c>
@@ -3942,7 +4022,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>281</v>
       </c>
@@ -3983,7 +4063,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>281</v>
       </c>
@@ -4024,7 +4104,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>281</v>
       </c>
@@ -4065,7 +4145,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>281</v>
       </c>
@@ -4106,7 +4186,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>281</v>
       </c>
@@ -4147,7 +4227,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>281</v>
       </c>
@@ -4188,7 +4268,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>281</v>
       </c>
@@ -4229,7 +4309,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>281</v>
       </c>
@@ -4270,7 +4350,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>281</v>
       </c>
@@ -4311,7 +4391,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>281</v>
       </c>
@@ -4352,7 +4432,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>281</v>
       </c>
@@ -4393,7 +4473,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>281</v>
       </c>
@@ -4434,7 +4514,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>348</v>
       </c>
@@ -4475,7 +4555,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>348</v>
       </c>
@@ -4516,7 +4596,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>348</v>
       </c>
@@ -4557,7 +4637,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>348</v>
       </c>
@@ -4598,7 +4678,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>348</v>
       </c>
@@ -4639,7 +4719,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>348</v>
       </c>
@@ -4680,7 +4760,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>348</v>
       </c>
@@ -4721,7 +4801,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>348</v>
       </c>
@@ -4762,7 +4842,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>348</v>
       </c>
@@ -4803,7 +4883,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>348</v>
       </c>
@@ -4844,7 +4924,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>348</v>
       </c>
@@ -4885,7 +4965,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>42</v>
       </c>
@@ -4926,7 +5006,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>42</v>
       </c>
@@ -4967,7 +5047,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>42</v>
       </c>
@@ -5008,7 +5088,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>42</v>
       </c>
@@ -5049,7 +5129,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>42</v>
       </c>
@@ -5090,7 +5170,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>42</v>
       </c>
@@ -5131,7 +5211,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>42</v>
       </c>
@@ -5172,7 +5252,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>42</v>
       </c>
@@ -5213,7 +5293,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>42</v>
       </c>
@@ -5254,7 +5334,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>42</v>
       </c>
@@ -5295,7 +5375,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>42</v>
       </c>
@@ -5336,7 +5416,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>42</v>
       </c>
@@ -5377,7 +5457,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>42</v>
       </c>
@@ -5418,7 +5498,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>42</v>
       </c>
@@ -5459,7 +5539,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>42</v>
       </c>
@@ -5500,7 +5580,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>42</v>
       </c>
@@ -5541,7 +5621,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>42</v>
       </c>
@@ -5582,7 +5662,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>42</v>
       </c>
@@ -5623,7 +5703,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>7</v>
       </c>
@@ -5664,7 +5744,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>7</v>
       </c>
@@ -5705,7 +5785,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>7</v>
       </c>
@@ -5746,7 +5826,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>7</v>
       </c>
@@ -5787,7 +5867,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>7</v>
       </c>
@@ -5828,7 +5908,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>7</v>
       </c>
@@ -5869,7 +5949,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>7</v>
       </c>
@@ -5910,7 +5990,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>7</v>
       </c>
@@ -5951,7 +6031,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>7</v>
       </c>
@@ -5992,7 +6072,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>7</v>
       </c>
@@ -6033,7 +6113,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>394</v>
       </c>
@@ -6074,7 +6154,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>394</v>
       </c>
@@ -6115,7 +6195,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>394</v>
       </c>
@@ -6156,7 +6236,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>394</v>
       </c>
@@ -6197,7 +6277,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>394</v>
       </c>
@@ -6238,7 +6318,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>394</v>
       </c>
@@ -6279,7 +6359,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>394</v>
       </c>
@@ -6320,7 +6400,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>394</v>
       </c>
@@ -6361,7 +6441,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>394</v>
       </c>
@@ -6402,7 +6482,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>394</v>
       </c>
@@ -6443,7 +6523,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>388</v>
       </c>
@@ -6486,10 +6566,20 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M112" xr:uid="{B6B4ECF6-20B5-45E9-BA32-692DD84773C2}">
-    <sortState ref="A2:M112">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M112">
       <sortCondition ref="F1:F112"/>
     </sortState>
   </autoFilter>
+  <mergeCells count="3">
+    <mergeCell ref="N2:N11"/>
+    <mergeCell ref="N12:N25"/>
+    <mergeCell ref="N26:N39"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{662D94E1-6FB0-4972-90EF-94B205ED028F}"/>
+    <hyperlink ref="N12" r:id="rId2" xr:uid="{04207750-D92E-4AAE-AB4E-876C45F423F2}"/>
+    <hyperlink ref="N26" r:id="rId3" xr:uid="{E41D56CF-94F1-4724-83FC-006E1E36D73D}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>